<commit_message>
Updates and new Scripts
</commit_message>
<xml_diff>
--- a/lithium_ion_batteries_statewide_20260903_123510.xlsx
+++ b/lithium_ion_batteries_statewide_20260903_123510.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ddion\Python Scripts\neris-toolbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30807DF0-EA58-472E-AC9D-3C34DC766B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D6D7FF1-9E42-4999-B1EB-ED1ED789A7A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Incident Details" sheetId="1" r:id="rId1"/>
@@ -2292,8 +2292,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="hh:mm"/>
-    <numFmt numFmtId="167" formatCode="m/d/yy;@"/>
+    <numFmt numFmtId="164" formatCode="hh:mm"/>
+    <numFmt numFmtId="165" formatCode="m/d/yy;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -2346,12 +2346,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2655,57 +2655,57 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AW95"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.36328125" customWidth="1"/>
+    <col min="2" max="2" width="39.42578125" customWidth="1"/>
     <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.90625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="42" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="69.90625" customWidth="1"/>
-    <col min="11" max="11" width="58.7265625" customWidth="1"/>
-    <col min="12" max="12" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="34.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.26953125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="48.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.90625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="64.453125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="40.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="69.85546875" customWidth="1"/>
+    <col min="11" max="11" width="58.7109375" customWidth="1"/>
+    <col min="12" max="12" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="48.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="40.140625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="39" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="78" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="25.7265625" customWidth="1"/>
-    <col min="31" max="31" width="32.26953125" customWidth="1"/>
-    <col min="32" max="32" width="49.6328125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="25.7109375" customWidth="1"/>
+    <col min="31" max="31" width="32.28515625" customWidth="1"/>
+    <col min="32" max="32" width="49.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="12" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="14" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="14" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:49" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2854,7 +2854,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -3006,7 +3006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>49</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>49</v>
       </c>
@@ -3228,7 +3228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -3304,7 +3304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>97</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>107</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>116</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>116</v>
       </c>
@@ -3678,7 +3678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>135</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>143</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>155</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>168</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>168</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>168</v>
       </c>
@@ -4140,7 +4140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>189</v>
       </c>
@@ -4216,7 +4216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>189</v>
       </c>
@@ -4292,7 +4292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>205</v>
       </c>
@@ -4371,7 +4371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>205</v>
       </c>
@@ -4450,7 +4450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>225</v>
       </c>
@@ -4520,7 +4520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>235</v>
       </c>
@@ -4593,7 +4593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>243</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>254</v>
       </c>
@@ -4739,7 +4739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>254</v>
       </c>
@@ -4815,7 +4815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>269</v>
       </c>
@@ -4894,7 +4894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>281</v>
       </c>
@@ -4973,7 +4973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>281</v>
       </c>
@@ -5046,7 +5046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>297</v>
       </c>
@@ -5122,7 +5122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>306</v>
       </c>
@@ -5198,7 +5198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>314</v>
       </c>
@@ -5271,7 +5271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>314</v>
       </c>
@@ -5350,7 +5350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>314</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>337</v>
       </c>
@@ -5499,7 +5499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>344</v>
       </c>
@@ -5575,7 +5575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>352</v>
       </c>
@@ -5651,7 +5651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>360</v>
       </c>
@@ -5721,7 +5721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>367</v>
       </c>
@@ -5800,7 +5800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>376</v>
       </c>
@@ -5870,7 +5870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>383</v>
       </c>
@@ -5940,7 +5940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>383</v>
       </c>
@@ -6010,7 +6010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>398</v>
       </c>
@@ -6089,7 +6089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>398</v>
       </c>
@@ -6168,7 +6168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>410</v>
       </c>
@@ -6244,7 +6244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>418</v>
       </c>
@@ -6323,7 +6323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>418</v>
       </c>
@@ -6402,7 +6402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>418</v>
       </c>
@@ -6481,7 +6481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>418</v>
       </c>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>418</v>
       </c>
@@ -6639,7 +6639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>418</v>
       </c>
@@ -6718,7 +6718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>418</v>
       </c>
@@ -6797,7 +6797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>418</v>
       </c>
@@ -6876,7 +6876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>418</v>
       </c>
@@ -6958,7 +6958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>418</v>
       </c>
@@ -7034,7 +7034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>418</v>
       </c>
@@ -7110,7 +7110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>469</v>
       </c>
@@ -7183,7 +7183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>469</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>469</v>
       </c>
@@ -7329,7 +7329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>487</v>
       </c>
@@ -7408,7 +7408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>487</v>
       </c>
@@ -7487,7 +7487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>498</v>
       </c>
@@ -7566,7 +7566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>498</v>
       </c>
@@ -7636,7 +7636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>512</v>
       </c>
@@ -7712,7 +7712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>512</v>
       </c>
@@ -7723,11 +7723,11 @@
         <v>521</v>
       </c>
       <c r="D66" s="5">
-        <f t="shared" ref="D66:D97" si="10">IF(C66="","",DATE(VALUE(LEFT(C66,4)),VALUE(MID(C66,6,2)),VALUE(MID(C66,9,2)))+TIME(VALUE(MID(C66,12,2)),VALUE(MID(C66,15,2)),VALUE(MID(C66,18,2)))-IF(AND(DATE(VALUE(LEFT(C66,4)),VALUE(MID(C66,6,2)),VALUE(MID(C66,9,2)))+TIME(VALUE(MID(C66,12,2)),VALUE(MID(C66,15,2)),VALUE(MID(C66,18,2)))&gt;=DATE(VALUE(LEFT(C66,4)),3,1)+MOD(8-WEEKDAY(DATE(VALUE(LEFT(C66,4)),3,1)),7)+7+TIME(7,0,0),DATE(VALUE(LEFT(C66,4)),3,1)+MOD(8-WEEKDAY(DATE(VALUE(LEFT(C66,4)),3,1)),7)+7+TIME(7,0,0)&lt;DATE(VALUE(LEFT(C66,4)),11,1)+MOD(8-WEEKDAY(DATE(VALUE(LEFT(C66,4)),11,1)),7)+TIME(6,0,0)), TIME(4,0,0),TIME(5,0,0)))</f>
+        <f t="shared" ref="D66:D95" si="10">IF(C66="","",DATE(VALUE(LEFT(C66,4)),VALUE(MID(C66,6,2)),VALUE(MID(C66,9,2)))+TIME(VALUE(MID(C66,12,2)),VALUE(MID(C66,15,2)),VALUE(MID(C66,18,2)))-IF(AND(DATE(VALUE(LEFT(C66,4)),VALUE(MID(C66,6,2)),VALUE(MID(C66,9,2)))+TIME(VALUE(MID(C66,12,2)),VALUE(MID(C66,15,2)),VALUE(MID(C66,18,2)))&gt;=DATE(VALUE(LEFT(C66,4)),3,1)+MOD(8-WEEKDAY(DATE(VALUE(LEFT(C66,4)),3,1)),7)+7+TIME(7,0,0),DATE(VALUE(LEFT(C66,4)),3,1)+MOD(8-WEEKDAY(DATE(VALUE(LEFT(C66,4)),3,1)),7)+7+TIME(7,0,0)&lt;DATE(VALUE(LEFT(C66,4)),11,1)+MOD(8-WEEKDAY(DATE(VALUE(LEFT(C66,4)),11,1)),7)+TIME(6,0,0)), TIME(4,0,0),TIME(5,0,0)))</f>
         <v>46065.184027777774</v>
       </c>
       <c r="E66" s="2">
-        <f t="shared" ref="E66:E97" si="11">IF(D66="","",MOD(D66,1))</f>
+        <f t="shared" ref="E66:E95" si="11">IF(D66="","",MOD(D66,1))</f>
         <v>0.18402777777373558</v>
       </c>
       <c r="F66">
@@ -7782,7 +7782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>527</v>
       </c>
@@ -7852,7 +7852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>534</v>
       </c>
@@ -7919,7 +7919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>534</v>
       </c>
@@ -7992,7 +7992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>547</v>
       </c>
@@ -8068,7 +8068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>547</v>
       </c>
@@ -8144,7 +8144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>558</v>
       </c>
@@ -8217,7 +8217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>558</v>
       </c>
@@ -8293,7 +8293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>558</v>
       </c>
@@ -8372,7 +8372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>558</v>
       </c>
@@ -8451,7 +8451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>558</v>
       </c>
@@ -8530,7 +8530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>586</v>
       </c>
@@ -8603,7 +8603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>586</v>
       </c>
@@ -8679,7 +8679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>598</v>
       </c>
@@ -8755,7 +8755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>606</v>
       </c>
@@ -8825,7 +8825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>613</v>
       </c>
@@ -8901,7 +8901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>623</v>
       </c>
@@ -8983,7 +8983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>623</v>
       </c>
@@ -9062,7 +9062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>637</v>
       </c>
@@ -9138,7 +9138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>644</v>
       </c>
@@ -9217,7 +9217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>654</v>
       </c>
@@ -9293,7 +9293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>662</v>
       </c>
@@ -9369,7 +9369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>669</v>
       </c>
@@ -9439,7 +9439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>676</v>
       </c>
@@ -9518,7 +9518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>684</v>
       </c>
@@ -9597,7 +9597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>692</v>
       </c>
@@ -9676,7 +9676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>700</v>
       </c>
@@ -9740,7 +9740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>705</v>
       </c>
@@ -9816,7 +9816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>712</v>
       </c>
@@ -9895,7 +9895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>719</v>
       </c>
@@ -9979,13 +9979,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>726</v>
       </c>
@@ -9993,7 +9993,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>728</v>
       </c>
@@ -10001,7 +10001,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>729</v>
       </c>
@@ -10009,7 +10009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>730</v>
       </c>
@@ -10017,7 +10017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>731</v>
       </c>
@@ -10025,7 +10025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>732</v>
       </c>
@@ -10033,7 +10033,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>733</v>
       </c>
@@ -10041,7 +10041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>734</v>
       </c>
@@ -10049,7 +10049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>735</v>
       </c>
@@ -10065,13 +10065,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="85" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>736</v>
       </c>
@@ -10079,7 +10079,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>738</v>
       </c>
@@ -10087,7 +10087,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>740</v>
       </c>
@@ -10095,7 +10095,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>742</v>
       </c>
@@ -10103,7 +10103,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>744</v>
       </c>
@@ -10111,7 +10111,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>746</v>
       </c>
@@ -10119,7 +10119,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>748</v>
       </c>

</xml_diff>